<commit_message>
improved cleanup (word-bounded enum match, unicode apostrophe, 80+ aliases) and 15-pass recheck producing manager Recoding Needed report
</commit_message>
<xml_diff>
--- a/Codebooks/Human Codebooks/content - cleaned/A - Content Analysis Codebook (cleaned) - Adanna.xlsx
+++ b/Codebooks/Human Codebooks/content - cleaned/A - Content Analysis Codebook (cleaned) - Adanna.xlsx
@@ -677,7 +677,7 @@
       <c r="F2" s="3" t="inlineStr"/>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Family/children, Social issues</t>
+          <t>Family/children, Social issues, e.g. corruption</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr"/>
@@ -710,7 +710,7 @@
       <c r="O2" s="3" t="inlineStr"/>
       <c r="P2" s="3" t="inlineStr">
         <is>
-          <t>Men's behavior, Mental health/emotional struggle</t>
+          <t>Mental health/emotional struggle, Men's behavior</t>
         </is>
       </c>
       <c r="Q2" s="3" t="inlineStr"/>
@@ -1046,7 +1046,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Been avoiding watching this Adolescence show on Netflix cos even the trailer is so triggering. 6 mins 39 secs in and I’ve had to pause. I’ve got 3 sons and know exactly how this will play out if it were me…</t>
+          <t>Been avoiding watching this Adolescence show on Netflix cos even the trailer is so triggering. 6 mins 39 secs in and I've had to pause. I've got 3 sons and know exactly how this will play out if it were me…</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -1058,7 +1058,7 @@
       <c r="F5" s="3" t="inlineStr"/>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Family/children, gender issues</t>
+          <t>Family/children, Gender issues, e.g. equality</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr"/>
@@ -1235,7 +1235,7 @@
       <c r="X6" s="3" t="inlineStr"/>
       <c r="Y6" s="3" t="inlineStr">
         <is>
-          <t>References external sources</t>
+          <t>References external sources, such as other influencers</t>
         </is>
       </c>
       <c r="Z6" s="3" t="inlineStr"/>
@@ -1354,7 +1354,7 @@
       <c r="X7" s="3" t="inlineStr"/>
       <c r="Y7" s="3" t="inlineStr">
         <is>
-          <t>Anecdotal exampled</t>
+          <t>Anecdotal examples</t>
         </is>
       </c>
       <c r="Z7" s="3" t="inlineStr"/>
@@ -1448,7 +1448,7 @@
       </c>
       <c r="P8" s="3" t="inlineStr">
         <is>
-          <t>Economic/status pressure, Men's behavior</t>
+          <t>Men's behavior, Economic/status pressure</t>
         </is>
       </c>
       <c r="Q8" s="3" t="inlineStr"/>
@@ -1534,7 +1534,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>GUYS ABEG ALWAYS ASK YOUR PPL HOW THEY ARE DOING, ESPECIALLY IF SOMETHING SEEMS OFF, AND DON’T SETTLE FOR “I’M FINE”!</t>
+          <t>GUYS ABEG ALWAYS ASK YOUR PPL HOW THEY ARE DOING, ESPECIALLY IF SOMETHING SEEMS OFF, AND DON'T SETTLE FOR "I'M FINE"!</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -1907,7 +1907,7 @@
       <c r="F12" s="3" t="inlineStr"/>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>Dating/marriage, Social issues, Religion/morality</t>
+          <t>Religion/morality, Dating/marriage, Social issues, e.g. corruption</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr"/>
@@ -2000,7 +2000,7 @@
       </c>
       <c r="AF12" s="3" t="inlineStr">
         <is>
-          <t>Calls for women to follow more equitable gender norms</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="AG12" s="3" t="inlineStr"/>
@@ -2057,7 +2057,7 @@
       </c>
       <c r="N13" s="3" t="inlineStr">
         <is>
-          <t>Not applicabe</t>
+          <t>Not applicable</t>
         </is>
       </c>
       <c r="O13" s="3" t="inlineStr"/>
@@ -2442,7 +2442,7 @@
       <c r="U16" s="3" t="inlineStr"/>
       <c r="V16" s="3" t="inlineStr">
         <is>
-          <t>Information seeking, Entertainment/escapism</t>
+          <t>Entertainment/escapism, Information seeking</t>
         </is>
       </c>
       <c r="W16" s="3" t="inlineStr">
@@ -2641,7 +2641,7 @@
       <c r="F18" s="3" t="inlineStr"/>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>Social issues, gender issues</t>
+          <t>Social issues, e.g. corruption, Gender issues, e.g. equality</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr"/>
@@ -3004,13 +3004,13 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>humor/sarcasm</t>
+          <t>Humor or sarcasm</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr"/>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>social issues</t>
+          <t>Social issues, e.g. corruption</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr"/>
@@ -3188,7 +3188,7 @@
       <c r="U22" s="3" t="inlineStr"/>
       <c r="V22" s="3" t="inlineStr">
         <is>
-          <t>Information seeking, Connection/social interaction</t>
+          <t>Connection/social interaction, Information seeking</t>
         </is>
       </c>
       <c r="W22" s="3" t="inlineStr">
@@ -3297,7 +3297,7 @@
       </c>
       <c r="P23" s="3" t="inlineStr">
         <is>
-          <t>Global political/social/cultural problems, Men's behavior, Women/feminism</t>
+          <t>Global political/social/cultural problems, Women/feminism, Men's behavior</t>
         </is>
       </c>
       <c r="Q23" s="3" t="inlineStr"/>
@@ -3315,7 +3315,7 @@
       <c r="U23" s="3" t="inlineStr"/>
       <c r="V23" s="3" t="inlineStr">
         <is>
-          <t>Information seeking, Entertainment/escapism</t>
+          <t>Entertainment/escapism, Information seeking</t>
         </is>
       </c>
       <c r="W23" s="3" t="inlineStr">
@@ -3326,7 +3326,7 @@
       <c r="X23" s="3" t="inlineStr"/>
       <c r="Y23" s="3" t="inlineStr">
         <is>
-          <t>Presented as common sense, References religion/tradition</t>
+          <t>References religion/tradition, Presented as common sense</t>
         </is>
       </c>
       <c r="Z23" s="3" t="inlineStr"/>
@@ -3357,7 +3357,7 @@
       </c>
       <c r="AF23" s="3" t="inlineStr">
         <is>
-          <t>Calls for men to follow more traditional gender norms</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="AG23" s="3" t="inlineStr"/>
@@ -3428,7 +3428,7 @@
       <c r="O24" s="3" t="inlineStr"/>
       <c r="P24" s="3" t="inlineStr">
         <is>
-          <t>Men's behavior, Women/feminism</t>
+          <t>Women/feminism, Men's behavior</t>
         </is>
       </c>
       <c r="Q24" s="3" t="inlineStr"/>
@@ -3541,13 +3541,13 @@
       </c>
       <c r="N25" s="3" t="inlineStr">
         <is>
-          <t>Men need to provide/succeed, Men need to improve themselves</t>
+          <t>Men need to improve themselves, Men need to provide/succeed</t>
         </is>
       </c>
       <c r="O25" s="3" t="inlineStr"/>
       <c r="P25" s="3" t="inlineStr">
         <is>
-          <t>Men's behavior, Global political/social/cultural problems</t>
+          <t>Global political/social/cultural problems, Men's behavior</t>
         </is>
       </c>
       <c r="Q25" s="3" t="inlineStr"/>
@@ -3565,7 +3565,7 @@
       <c r="U25" s="3" t="inlineStr"/>
       <c r="V25" s="3" t="inlineStr">
         <is>
-          <t>Information seeking, Connection/social interaction</t>
+          <t>Connection/social interaction, Information seeking</t>
         </is>
       </c>
       <c r="W25" s="3" t="inlineStr">
@@ -3678,7 +3678,7 @@
       <c r="O26" s="3" t="inlineStr"/>
       <c r="P26" s="3" t="inlineStr">
         <is>
-          <t>Men's behavior, Women/feminism</t>
+          <t>Women/feminism, Men's behavior</t>
         </is>
       </c>
       <c r="Q26" s="3" t="inlineStr"/>
@@ -3815,7 +3815,7 @@
       <c r="U27" s="3" t="inlineStr"/>
       <c r="V27" s="3" t="inlineStr">
         <is>
-          <t>Information seeking, Connection/social interaction</t>
+          <t>Connection/social interaction, Information seeking</t>
         </is>
       </c>
       <c r="W27" s="3" t="inlineStr">
@@ -3938,7 +3938,7 @@
       <c r="U28" s="3" t="inlineStr"/>
       <c r="V28" s="3" t="inlineStr">
         <is>
-          <t>Information seeking, Connection/social interaction</t>
+          <t>Connection/social interaction, Information seeking</t>
         </is>
       </c>
       <c r="W28" s="3" t="inlineStr">
@@ -4033,13 +4033,13 @@
       </c>
       <c r="N29" s="3" t="inlineStr">
         <is>
-          <t>Men need to improve themselves, Men need to dominate/ead</t>
+          <t>Men need to improve themselves, Men need to dominate/lead</t>
         </is>
       </c>
       <c r="O29" s="3" t="inlineStr"/>
       <c r="P29" s="3" t="inlineStr">
         <is>
-          <t>Men's behavior, Global political/social/cultural problems</t>
+          <t>Global political/social/cultural problems, Men's behavior</t>
         </is>
       </c>
       <c r="Q29" s="3" t="inlineStr"/>
@@ -4057,7 +4057,7 @@
       <c r="U29" s="3" t="inlineStr"/>
       <c r="V29" s="3" t="inlineStr">
         <is>
-          <t>Information seeking, Connection/social interaction</t>
+          <t>Connection/social interaction, Information seeking</t>
         </is>
       </c>
       <c r="W29" s="3" t="inlineStr">
@@ -4133,7 +4133,7 @@
       <c r="F30" s="3" t="inlineStr"/>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>Dating/marriage, Social issues</t>
+          <t>Dating/marriage, Social issues, e.g. corruption</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr"/>
@@ -4252,7 +4252,7 @@
       <c r="F31" s="3" t="inlineStr"/>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>Dating/marriage, Gaming/technology</t>
+          <t>Gaming/technology, Dating/marriage</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr"/>
@@ -4303,7 +4303,7 @@
       <c r="U31" s="3" t="inlineStr"/>
       <c r="V31" s="3" t="inlineStr">
         <is>
-          <t>Information seeking, Connection/social interaction</t>
+          <t>Connection/social interaction, Information seeking</t>
         </is>
       </c>
       <c r="W31" s="3" t="inlineStr">
@@ -4412,7 +4412,7 @@
       <c r="O32" s="3" t="inlineStr"/>
       <c r="P32" s="3" t="inlineStr">
         <is>
-          <t>Men's behavior, Women/feminism</t>
+          <t>Women/feminism, Men's behavior</t>
         </is>
       </c>
       <c r="Q32" s="3" t="inlineStr"/>
@@ -4424,7 +4424,7 @@
       <c r="S32" s="3" t="inlineStr"/>
       <c r="T32" s="3" t="inlineStr">
         <is>
-          <t>Commenary/opinion</t>
+          <t>Commentary/opinion</t>
         </is>
       </c>
       <c r="U32" s="3" t="inlineStr"/>
@@ -4498,7 +4498,7 @@
       <c r="F33" s="3" t="inlineStr"/>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>Gender issues, social issues, Dating/marriage</t>
+          <t>Dating/marriage, Gender issues, e.g. equality, Social issues, e.g. corruption</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr"/>
@@ -4549,7 +4549,7 @@
       <c r="U33" s="3" t="inlineStr"/>
       <c r="V33" s="3" t="inlineStr">
         <is>
-          <t>Information seeking, Connection/social interaction</t>
+          <t>Connection/social interaction, Information seeking</t>
         </is>
       </c>
       <c r="W33" s="3" t="inlineStr">
@@ -4617,7 +4617,7 @@
       <c r="F34" s="3" t="inlineStr"/>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>Gender issues, social issues</t>
+          <t>Gender issues, e.g. equality, Social issues, e.g. corruption</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr"/>
@@ -4650,7 +4650,7 @@
       <c r="O34" s="3" t="inlineStr"/>
       <c r="P34" s="3" t="inlineStr">
         <is>
-          <t>Men's behavior, Global political/social/cultural problems</t>
+          <t>Global political/social/cultural problems, Men's behavior</t>
         </is>
       </c>
       <c r="Q34" s="3" t="inlineStr"/>
@@ -4662,7 +4662,7 @@
       <c r="S34" s="3" t="inlineStr"/>
       <c r="T34" s="3" t="inlineStr">
         <is>
-          <t>Personal story, Commentary/opinion</t>
+          <t>Commentary/opinion, Personal story</t>
         </is>
       </c>
       <c r="U34" s="3" t="inlineStr"/>
@@ -4769,7 +4769,7 @@
       <c r="O35" s="3" t="inlineStr"/>
       <c r="P35" s="3" t="inlineStr">
         <is>
-          <t>Men's behavior, Women/feminism, Global political/social/cultural problems</t>
+          <t>Global political/social/cultural problems, Women/feminism, Men's behavior</t>
         </is>
       </c>
       <c r="Q35" s="3" t="inlineStr"/>
@@ -4785,13 +4785,13 @@
       </c>
       <c r="T35" s="3" t="inlineStr">
         <is>
-          <t>Personal story, Commentary/opinion</t>
+          <t>Commentary/opinion, Personal story</t>
         </is>
       </c>
       <c r="U35" s="3" t="inlineStr"/>
       <c r="V35" s="3" t="inlineStr">
         <is>
-          <t>Information seeking, Connection/social interaction</t>
+          <t>Connection/social interaction, Information seeking</t>
         </is>
       </c>
       <c r="W35" s="3" t="inlineStr">
@@ -4910,7 +4910,7 @@
       <c r="U36" s="3" t="inlineStr"/>
       <c r="V36" s="3" t="inlineStr">
         <is>
-          <t>Information seeking, Entertainment/escapism</t>
+          <t>Entertainment/escapism, Information seeking</t>
         </is>
       </c>
       <c r="W36" s="3" t="inlineStr">
@@ -4978,7 +4978,7 @@
       <c r="F37" s="3" t="inlineStr"/>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>Dating/marriage, Gender issues</t>
+          <t>Dating/marriage, Gender issues, e.g. equality</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr"/>
@@ -5160,7 +5160,7 @@
       </c>
       <c r="V38" s="3" t="inlineStr">
         <is>
-          <t>Information seeking, Connection/social interaction</t>
+          <t>Connection/social interaction, Information seeking</t>
         </is>
       </c>
       <c r="W38" s="3" t="inlineStr">
@@ -5263,7 +5263,7 @@
       </c>
       <c r="N39" s="3" t="inlineStr">
         <is>
-          <t>Men need to be more emotionally open</t>
+          <t>Men need to be emotionally open</t>
         </is>
       </c>
       <c r="O39" s="3" t="inlineStr"/>
@@ -5281,13 +5281,13 @@
       <c r="S39" s="3" t="inlineStr"/>
       <c r="T39" s="3" t="inlineStr">
         <is>
-          <t>Advice/instruction, Personal story, Commentary/opinion</t>
+          <t>Advice/instruction, Commentary/opinion, Personal story</t>
         </is>
       </c>
       <c r="U39" s="3" t="inlineStr"/>
       <c r="V39" s="3" t="inlineStr">
         <is>
-          <t>Information seeking, Entertainment/escapism</t>
+          <t>Entertainment/escapism, Information seeking</t>
         </is>
       </c>
       <c r="W39" s="3" t="inlineStr">
@@ -5396,7 +5396,7 @@
       <c r="O40" s="3" t="inlineStr"/>
       <c r="P40" s="3" t="inlineStr">
         <is>
-          <t>Economic/status pressure, Global political/social/cultural problems</t>
+          <t>Global political/social/cultural problems, Economic/status pressure</t>
         </is>
       </c>
       <c r="Q40" s="3" t="inlineStr"/>
@@ -5862,7 +5862,7 @@
       <c r="O2" s="3" t="inlineStr"/>
       <c r="P2" s="3" t="inlineStr">
         <is>
-          <t>Men's behavior, Economic/status pressure</t>
+          <t>Economic/status pressure, Men's behavior</t>
         </is>
       </c>
       <c r="Q2" s="3" t="inlineStr"/>
@@ -5880,7 +5880,7 @@
       <c r="U2" s="3" t="inlineStr"/>
       <c r="V2" s="3" t="inlineStr">
         <is>
-          <t>Information seeking, Connection/social interaction</t>
+          <t>Connection/social interaction, Information seeking</t>
         </is>
       </c>
       <c r="W2" s="3" t="inlineStr">
@@ -5948,7 +5948,7 @@
       <c r="F3" s="3" t="inlineStr"/>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Dating/marriage, Social issues</t>
+          <t>Dating/marriage, Social issues, e.g. corruption</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr"/>
@@ -6227,7 +6227,7 @@
       <c r="O5" s="3" t="inlineStr"/>
       <c r="P5" s="3" t="inlineStr">
         <is>
-          <t>Men's behavior, Economic/status pressure</t>
+          <t>Economic/status pressure, Men's behavior</t>
         </is>
       </c>
       <c r="Q5" s="3" t="inlineStr"/>
@@ -6346,7 +6346,7 @@
       <c r="O6" s="3" t="inlineStr"/>
       <c r="P6" s="3" t="inlineStr">
         <is>
-          <t>Men's behavior, Mental health/emotional struggle</t>
+          <t>Mental health/emotional struggle, Men's behavior</t>
         </is>
       </c>
       <c r="Q6" s="3" t="inlineStr"/>
@@ -6551,7 +6551,7 @@
       <c r="F8" s="3" t="inlineStr"/>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Mental health, gender issues</t>
+          <t>Mental health, Gender issues, e.g. equality</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr"/>
@@ -6584,7 +6584,7 @@
       <c r="O8" s="3" t="inlineStr"/>
       <c r="P8" s="3" t="inlineStr">
         <is>
-          <t>Men's behavior, Mental health/emotional struggle</t>
+          <t>Mental health/emotional struggle, Men's behavior</t>
         </is>
       </c>
       <c r="Q8" s="3" t="inlineStr"/>
@@ -6682,7 +6682,7 @@
       <c r="F9" s="3" t="inlineStr"/>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Mental health, gender issues</t>
+          <t>Mental health, Gender issues, e.g. equality</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr"/>
@@ -6715,7 +6715,7 @@
       <c r="O9" s="3" t="inlineStr"/>
       <c r="P9" s="3" t="inlineStr">
         <is>
-          <t>Men's behavior, Mental health/emotional struggle</t>
+          <t>Mental health/emotional struggle, Men's behavior</t>
         </is>
       </c>
       <c r="Q9" s="3" t="inlineStr"/>
@@ -6801,7 +6801,7 @@
       <c r="F10" s="3" t="inlineStr"/>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>Mental health, gender issues</t>
+          <t>Mental health, Gender issues, e.g. equality</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr"/>
@@ -6838,7 +6838,7 @@
       </c>
       <c r="P10" s="3" t="inlineStr">
         <is>
-          <t>Men's behavior, Mental health/emotional struggle</t>
+          <t>Mental health/emotional struggle, Men's behavior</t>
         </is>
       </c>
       <c r="Q10" s="3" t="inlineStr"/>
@@ -6928,7 +6928,7 @@
       <c r="F11" s="3" t="inlineStr"/>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>Gender issues, social issues, Mental health</t>
+          <t>Mental health, Gender issues, e.g. equality, Social issues, e.g. corruption</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr"/>
@@ -6961,7 +6961,7 @@
       <c r="O11" s="3" t="inlineStr"/>
       <c r="P11" s="3" t="inlineStr">
         <is>
-          <t>Men's behavior, Mental health/emotional struggle</t>
+          <t>Mental health/emotional struggle, Men's behavior</t>
         </is>
       </c>
       <c r="Q11" s="3" t="inlineStr"/>
@@ -7047,7 +7047,7 @@
       <c r="F12" s="3" t="inlineStr"/>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>Gender issues, social issues</t>
+          <t>Gender issues, e.g. equality, Social issues, e.g. corruption</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr"/>
@@ -7166,7 +7166,7 @@
       <c r="F13" s="3" t="inlineStr"/>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>Gender issues, social issues</t>
+          <t>Gender issues, e.g. equality, Social issues, e.g. corruption</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr"/>
@@ -7285,7 +7285,7 @@
       <c r="F14" s="3" t="inlineStr"/>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>Gender issues, social issues, Dating/marriage</t>
+          <t>Dating/marriage, Gender issues, e.g. equality, Social issues, e.g. corruption</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr"/>
@@ -7404,7 +7404,7 @@
       <c r="F15" s="3" t="inlineStr"/>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>Gender issues, social issues, Dating/marriage</t>
+          <t>Dating/marriage, Gender issues, e.g. equality, Social issues, e.g. corruption</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr"/>
@@ -7523,7 +7523,7 @@
       <c r="F16" s="3" t="inlineStr"/>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>Social issues</t>
+          <t>Social issues, e.g. corruption</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr"/>
@@ -7579,7 +7579,7 @@
       </c>
       <c r="W16" s="3" t="inlineStr">
         <is>
-          <t>Anecdotal examples</t>
+          <t>Personal experience</t>
         </is>
       </c>
       <c r="X16" s="3" t="inlineStr"/>
@@ -7739,7 +7739,7 @@
       </c>
       <c r="AF17" s="3" t="inlineStr">
         <is>
-          <t>Dominate more</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="AG17" s="3" t="inlineStr"/>
@@ -7777,7 +7777,7 @@
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>Gender issues</t>
+          <t>Gender issues, e.g. equality</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr"/>
@@ -7927,7 +7927,7 @@
       </c>
       <c r="N19" s="3" t="inlineStr">
         <is>
-          <t>Men need to dominate/ead</t>
+          <t>Men need to dominate/lead</t>
         </is>
       </c>
       <c r="O19" s="3" t="inlineStr"/>
@@ -7993,7 +7993,7 @@
       </c>
       <c r="AF19" s="3" t="inlineStr">
         <is>
-          <t>Dominate more</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="AG19" s="3" t="inlineStr"/>
@@ -8027,7 +8027,7 @@
       <c r="F20" s="3" t="inlineStr"/>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>Gender issues, social issues</t>
+          <t>Gender issues, e.g. equality, Social issues, e.g. corruption</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr"/>
@@ -8146,7 +8146,7 @@
       <c r="F21" s="3" t="inlineStr"/>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>Gender issues</t>
+          <t>Gender issues, e.g. equality</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr"/>
@@ -8316,7 +8316,7 @@
       <c r="U22" s="3" t="inlineStr"/>
       <c r="V22" s="3" t="inlineStr">
         <is>
-          <t>Information seeking, connetion/social interaction</t>
+          <t>Information seeking, Connection/social interaction</t>
         </is>
       </c>
       <c r="W22" s="3" t="inlineStr">
@@ -8415,7 +8415,7 @@
       </c>
       <c r="N23" s="3" t="inlineStr">
         <is>
-          <t>Men need to now show emotions</t>
+          <t>Men need to not show emotions</t>
         </is>
       </c>
       <c r="O23" s="3" t="inlineStr"/>
@@ -8433,13 +8433,13 @@
       <c r="S23" s="3" t="inlineStr"/>
       <c r="T23" s="3" t="inlineStr">
         <is>
-          <t>Personal story, Commentary/opinion</t>
+          <t>Commentary/opinion, Personal story</t>
         </is>
       </c>
       <c r="U23" s="3" t="inlineStr"/>
       <c r="V23" s="3" t="inlineStr">
         <is>
-          <t>Information seeking, connetion/social interaction</t>
+          <t>Information seeking, Connection/social interaction</t>
         </is>
       </c>
       <c r="W23" s="3" t="inlineStr">
@@ -8534,13 +8534,13 @@
       </c>
       <c r="N24" s="3" t="inlineStr">
         <is>
-          <t>Men need to dominate/lead, Men need to now show emotions</t>
+          <t>Men need to dominate/lead, Men need to not show emotions</t>
         </is>
       </c>
       <c r="O24" s="3" t="inlineStr"/>
       <c r="P24" s="3" t="inlineStr">
         <is>
-          <t>Men's behavior, Women/feminism</t>
+          <t>Women/feminism, Men's behavior</t>
         </is>
       </c>
       <c r="Q24" s="3" t="inlineStr"/>
@@ -8558,7 +8558,7 @@
       <c r="U24" s="3" t="inlineStr"/>
       <c r="V24" s="3" t="inlineStr">
         <is>
-          <t>Information seeking, connetion/social interaction</t>
+          <t>Information seeking, Connection/social interaction</t>
         </is>
       </c>
       <c r="W24" s="3" t="inlineStr">
@@ -8600,7 +8600,7 @@
       </c>
       <c r="AF24" s="3" t="inlineStr">
         <is>
-          <t>Calls for men to follow more traditional gender norms</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="AG24" s="3" t="inlineStr"/>
@@ -8681,7 +8681,7 @@
       <c r="U25" s="3" t="inlineStr"/>
       <c r="V25" s="3" t="inlineStr">
         <is>
-          <t>Information seeking, connetion/social interaction</t>
+          <t>Information seeking, Connection/social interaction</t>
         </is>
       </c>
       <c r="W25" s="3" t="inlineStr">
@@ -8723,7 +8723,7 @@
       </c>
       <c r="AF25" s="3" t="inlineStr">
         <is>
-          <t>Calls for men to follow more traditional gender norms</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="AG25" s="3" t="inlineStr"/>
@@ -8812,7 +8812,7 @@
       <c r="U26" s="3" t="inlineStr"/>
       <c r="V26" s="3" t="inlineStr">
         <is>
-          <t>Information seeking, connetion/social interaction</t>
+          <t>Information seeking, Connection/social interaction</t>
         </is>
       </c>
       <c r="W26" s="3" t="inlineStr">
@@ -8854,7 +8854,7 @@
       </c>
       <c r="AF26" s="3" t="inlineStr">
         <is>
-          <t>Calls for men to follow more traditional gender norms</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="AG26" s="3" t="inlineStr"/>
@@ -8882,7 +8882,7 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>Uses all CAPS</t>
+          <t>Use of all CAPS</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr"/>
@@ -8915,19 +8915,19 @@
       </c>
       <c r="N27" s="3" t="inlineStr">
         <is>
-          <t>Men need to dominate/lead, Men need to improve themselves, Men need to be fully self-reliant</t>
+          <t>Men need to be fully self-reliant, Men need to improve themselves, Men need to dominate/lead</t>
         </is>
       </c>
       <c r="O27" s="3" t="inlineStr"/>
       <c r="P27" s="3" t="inlineStr">
         <is>
-          <t>Men's behavior, Women/feminism</t>
+          <t>Women/feminism, Men's behavior</t>
         </is>
       </c>
       <c r="Q27" s="3" t="inlineStr"/>
       <c r="R27" s="3" t="inlineStr">
         <is>
-          <t>Assert dominance/control, More self-discipline/fitness</t>
+          <t>More self-discipline/fitness, Assert dominance/control</t>
         </is>
       </c>
       <c r="S27" s="3" t="inlineStr"/>
@@ -8939,7 +8939,7 @@
       <c r="U27" s="3" t="inlineStr"/>
       <c r="V27" s="3" t="inlineStr">
         <is>
-          <t>Information seeking, connetion/social interaction</t>
+          <t>Information seeking, Connection/social interaction</t>
         </is>
       </c>
       <c r="W27" s="3" t="inlineStr">
@@ -8981,7 +8981,7 @@
       </c>
       <c r="AF27" s="3" t="inlineStr">
         <is>
-          <t>Calls for men to follow more traditional gender norms</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="AG27" s="3" t="inlineStr"/>
@@ -9044,7 +9044,7 @@
       <c r="O28" s="3" t="inlineStr"/>
       <c r="P28" s="3" t="inlineStr">
         <is>
-          <t>Men's behavior, Women/feminism</t>
+          <t>Women/feminism, Men's behavior</t>
         </is>
       </c>
       <c r="Q28" s="3" t="inlineStr"/>
@@ -9062,7 +9062,7 @@
       <c r="U28" s="3" t="inlineStr"/>
       <c r="V28" s="3" t="inlineStr">
         <is>
-          <t>Information seeking, connetion/social interaction</t>
+          <t>Information seeking, Connection/social interaction</t>
         </is>
       </c>
       <c r="W28" s="3" t="inlineStr">
@@ -9104,7 +9104,7 @@
       </c>
       <c r="AF28" s="3" t="inlineStr">
         <is>
-          <t>Calls for men to follow more traditional gender norms</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="AG28" s="3" t="inlineStr"/>
@@ -9185,7 +9185,7 @@
       <c r="U29" s="3" t="inlineStr"/>
       <c r="V29" s="3" t="inlineStr">
         <is>
-          <t>Information seeking, connetion/social interaction</t>
+          <t>Information seeking, Connection/social interaction</t>
         </is>
       </c>
       <c r="W29" s="3" t="inlineStr">
@@ -9227,7 +9227,7 @@
       </c>
       <c r="AF29" s="3" t="inlineStr">
         <is>
-          <t>Calls for men to follow more traditional gender norms</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="AG29" s="3" t="inlineStr"/>
@@ -9257,7 +9257,7 @@
       <c r="F30" s="3" t="inlineStr"/>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>Gender issues, social issues</t>
+          <t>Gender issues, e.g. equality, Social issues, e.g. corruption</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr"/>
@@ -9294,7 +9294,7 @@
       </c>
       <c r="P30" s="3" t="inlineStr">
         <is>
-          <t>Men's behavior, Global political/social/cultural problems</t>
+          <t>Global political/social/cultural problems, Men's behavior</t>
         </is>
       </c>
       <c r="Q30" s="3" t="inlineStr"/>
@@ -9312,7 +9312,7 @@
       <c r="U30" s="3" t="inlineStr"/>
       <c r="V30" s="3" t="inlineStr">
         <is>
-          <t>Information seeking, connetion/social interaction</t>
+          <t>Information seeking, Connection/social interaction</t>
         </is>
       </c>
       <c r="W30" s="3" t="inlineStr">
@@ -9323,7 +9323,7 @@
       <c r="X30" s="3" t="inlineStr"/>
       <c r="Y30" s="3" t="inlineStr">
         <is>
-          <t>References external sources</t>
+          <t>References external sources, such as other influencers</t>
         </is>
       </c>
       <c r="Z30" s="3" t="inlineStr"/>
@@ -9388,7 +9388,7 @@
       <c r="F31" s="3" t="inlineStr"/>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>Gender issues, social issues</t>
+          <t>Gender issues, e.g. equality, Social issues, e.g. corruption</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr"/>
@@ -9425,7 +9425,7 @@
       </c>
       <c r="P31" s="3" t="inlineStr">
         <is>
-          <t>Men's behavior, Global political/social/cultural problems</t>
+          <t>Global political/social/cultural problems, Men's behavior</t>
         </is>
       </c>
       <c r="Q31" s="3" t="inlineStr"/>
@@ -9443,7 +9443,7 @@
       <c r="U31" s="3" t="inlineStr"/>
       <c r="V31" s="3" t="inlineStr">
         <is>
-          <t>Information seeking, connetion/social interaction</t>
+          <t>Information seeking, Connection/social interaction</t>
         </is>
       </c>
       <c r="W31" s="3" t="inlineStr">
@@ -9570,7 +9570,7 @@
       <c r="U32" s="3" t="inlineStr"/>
       <c r="V32" s="3" t="inlineStr">
         <is>
-          <t>Information seeking, connetion/social interaction</t>
+          <t>Information seeking, Connection/social interaction</t>
         </is>
       </c>
       <c r="W32" s="3" t="inlineStr">
@@ -9612,7 +9612,7 @@
       </c>
       <c r="AF32" s="3" t="inlineStr">
         <is>
-          <t>Calls for men to follow more traditional gender norms</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="AG32" s="3" t="inlineStr"/>
@@ -9735,7 +9735,7 @@
       </c>
       <c r="AF33" s="3" t="inlineStr">
         <is>
-          <t>Calls for men to follow more traditional gender norms</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="AG33" s="3" t="inlineStr"/>
@@ -10011,7 +10011,7 @@
       <c r="F36" s="3" t="inlineStr"/>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>Gender issues</t>
+          <t>Gender issues, e.g. equality</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr"/>
@@ -10050,7 +10050,7 @@
       <c r="Q36" s="3" t="inlineStr"/>
       <c r="R36" s="3" t="inlineStr">
         <is>
-          <t>Social or political change, More emotional growth/healing</t>
+          <t>More emotional growth/healing, Social or political change</t>
         </is>
       </c>
       <c r="S36" s="3" t="inlineStr"/>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="AF36" s="3" t="inlineStr">
         <is>
-          <t>Calls for men to follow more equitable gender norms</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="AG36" s="3" t="inlineStr"/>
@@ -10167,13 +10167,13 @@
       <c r="O37" s="3" t="inlineStr"/>
       <c r="P37" s="3" t="inlineStr">
         <is>
-          <t>Men's behavior, Women/feminism</t>
+          <t>Women/feminism, Men's behavior</t>
         </is>
       </c>
       <c r="Q37" s="3" t="inlineStr"/>
       <c r="R37" s="3" t="inlineStr">
         <is>
-          <t>Assert dominance/control, More equality/respect for women</t>
+          <t>More equality/respect for women, Assert dominance/control</t>
         </is>
       </c>
       <c r="S37" s="3" t="inlineStr"/>
@@ -10185,7 +10185,7 @@
       <c r="U37" s="3" t="inlineStr"/>
       <c r="V37" s="3" t="inlineStr">
         <is>
-          <t>Information seeking, Connection/social interaction</t>
+          <t>Connection/social interaction, Information seeking</t>
         </is>
       </c>
       <c r="W37" s="3" t="inlineStr">
@@ -10269,7 +10269,7 @@
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>Mental health, Dating/marriage</t>
+          <t>Dating/marriage, Mental health</t>
         </is>
       </c>
       <c r="H38" s="3" t="inlineStr"/>
@@ -10366,7 +10366,7 @@
       </c>
       <c r="AF38" s="3" t="inlineStr">
         <is>
-          <t>Calls for men to follow more traditional gender norms</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="AG38" s="3" t="inlineStr"/>
@@ -10396,7 +10396,7 @@
       <c r="F39" s="3" t="inlineStr"/>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>Mental heath</t>
+          <t>Mental health</t>
         </is>
       </c>
       <c r="H39" s="3" t="inlineStr"/>
@@ -10556,7 +10556,7 @@
       <c r="O40" s="3" t="inlineStr"/>
       <c r="P40" s="3" t="inlineStr">
         <is>
-          <t>Men's behavior, Women/feminism</t>
+          <t>Women/feminism, Men's behavior</t>
         </is>
       </c>
       <c r="Q40" s="3" t="inlineStr"/>
@@ -10574,7 +10574,7 @@
       <c r="U40" s="3" t="inlineStr"/>
       <c r="V40" s="3" t="inlineStr">
         <is>
-          <t>Information seeking, Connection/social interaction</t>
+          <t>Connection/social interaction, Information seeking</t>
         </is>
       </c>
       <c r="W40" s="3" t="inlineStr">
@@ -10616,7 +10616,7 @@
       </c>
       <c r="AF40" s="3" t="inlineStr">
         <is>
-          <t>Calls for men to follow more traditional gender norms</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="AG40" s="3" t="inlineStr"/>
@@ -10646,7 +10646,7 @@
       <c r="F41" s="3" t="inlineStr"/>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>Mental health, Fitness/self-improvement</t>
+          <t>Fitness/self-improvement, Mental health</t>
         </is>
       </c>
       <c r="H41" s="3" t="inlineStr"/>

</xml_diff>

<commit_message>
fix recheck script: None-string bug inflated Q4/Q5 contradictions (4 real not 41); stop auto-mapping invented Q18a categories to Other (which made cleanup artifacts look like coder errors)
</commit_message>
<xml_diff>
--- a/Codebooks/Human Codebooks/content - cleaned/A - Content Analysis Codebook (cleaned) - Adanna.xlsx
+++ b/Codebooks/Human Codebooks/content - cleaned/A - Content Analysis Codebook (cleaned) - Adanna.xlsx
@@ -2000,7 +2000,7 @@
       </c>
       <c r="AF12" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Calls for women to follow more equitable gender norms</t>
         </is>
       </c>
       <c r="AG12" s="3" t="inlineStr"/>
@@ -3357,7 +3357,7 @@
       </c>
       <c r="AF23" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Calls for men to follow more traditional gender norms</t>
         </is>
       </c>
       <c r="AG23" s="3" t="inlineStr"/>
@@ -7739,7 +7739,7 @@
       </c>
       <c r="AF17" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Dominate more</t>
         </is>
       </c>
       <c r="AG17" s="3" t="inlineStr"/>
@@ -7993,7 +7993,7 @@
       </c>
       <c r="AF19" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Dominate more</t>
         </is>
       </c>
       <c r="AG19" s="3" t="inlineStr"/>
@@ -8600,7 +8600,7 @@
       </c>
       <c r="AF24" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Calls for men to follow more traditional gender norms</t>
         </is>
       </c>
       <c r="AG24" s="3" t="inlineStr"/>
@@ -8723,7 +8723,7 @@
       </c>
       <c r="AF25" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Calls for men to follow more traditional gender norms</t>
         </is>
       </c>
       <c r="AG25" s="3" t="inlineStr"/>
@@ -8854,7 +8854,7 @@
       </c>
       <c r="AF26" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Calls for men to follow more traditional gender norms</t>
         </is>
       </c>
       <c r="AG26" s="3" t="inlineStr"/>
@@ -8981,7 +8981,7 @@
       </c>
       <c r="AF27" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Calls for men to follow more traditional gender norms</t>
         </is>
       </c>
       <c r="AG27" s="3" t="inlineStr"/>
@@ -9104,7 +9104,7 @@
       </c>
       <c r="AF28" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Calls for men to follow more traditional gender norms</t>
         </is>
       </c>
       <c r="AG28" s="3" t="inlineStr"/>
@@ -9227,7 +9227,7 @@
       </c>
       <c r="AF29" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Calls for men to follow more traditional gender norms</t>
         </is>
       </c>
       <c r="AG29" s="3" t="inlineStr"/>
@@ -9612,7 +9612,7 @@
       </c>
       <c r="AF32" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Calls for men to follow more traditional gender norms</t>
         </is>
       </c>
       <c r="AG32" s="3" t="inlineStr"/>
@@ -9735,7 +9735,7 @@
       </c>
       <c r="AF33" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Calls for men to follow more traditional gender norms</t>
         </is>
       </c>
       <c r="AG33" s="3" t="inlineStr"/>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="AF36" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Calls for men to follow more equitable gender norms</t>
         </is>
       </c>
       <c r="AG36" s="3" t="inlineStr"/>
@@ -10366,7 +10366,7 @@
       </c>
       <c r="AF38" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Calls for men to follow more traditional gender norms</t>
         </is>
       </c>
       <c r="AG38" s="3" t="inlineStr"/>
@@ -10616,7 +10616,7 @@
       </c>
       <c r="AF40" s="3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Calls for men to follow more traditional gender norms</t>
         </is>
       </c>
       <c r="AG40" s="3" t="inlineStr"/>

</xml_diff>

<commit_message>
unified processor: clean both content + audience codebooks, build master files and recoding action list
</commit_message>
<xml_diff>
--- a/Codebooks/Human Codebooks/content - cleaned/A - Content Analysis Codebook (cleaned) - Adanna.xlsx
+++ b/Codebooks/Human Codebooks/content - cleaned/A - Content Analysis Codebook (cleaned) - Adanna.xlsx
@@ -450,42 +450,42 @@
   <dimension ref="A1:AG41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="45" customWidth="1" min="2" max="2"/>
-    <col width="45" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
-    <col width="28" customWidth="1" min="8" max="8"/>
-    <col width="28" customWidth="1" min="9" max="9"/>
-    <col width="28" customWidth="1" min="10" max="10"/>
-    <col width="28" customWidth="1" min="11" max="11"/>
-    <col width="28" customWidth="1" min="12" max="12"/>
-    <col width="28" customWidth="1" min="13" max="13"/>
-    <col width="28" customWidth="1" min="14" max="14"/>
-    <col width="28" customWidth="1" min="15" max="15"/>
-    <col width="28" customWidth="1" min="16" max="16"/>
-    <col width="28" customWidth="1" min="17" max="17"/>
-    <col width="28" customWidth="1" min="18" max="18"/>
-    <col width="28" customWidth="1" min="19" max="19"/>
-    <col width="28" customWidth="1" min="20" max="20"/>
-    <col width="28" customWidth="1" min="21" max="21"/>
-    <col width="28" customWidth="1" min="22" max="22"/>
-    <col width="28" customWidth="1" min="23" max="23"/>
-    <col width="28" customWidth="1" min="24" max="24"/>
-    <col width="28" customWidth="1" min="25" max="25"/>
-    <col width="28" customWidth="1" min="26" max="26"/>
-    <col width="28" customWidth="1" min="27" max="27"/>
-    <col width="28" customWidth="1" min="28" max="28"/>
-    <col width="28" customWidth="1" min="29" max="29"/>
-    <col width="28" customWidth="1" min="30" max="30"/>
-    <col width="28" customWidth="1" min="31" max="31"/>
-    <col width="28" customWidth="1" min="32" max="32"/>
-    <col width="28" customWidth="1" min="33" max="33"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="13" max="13"/>
+    <col width="26" customWidth="1" min="14" max="14"/>
+    <col width="26" customWidth="1" min="15" max="15"/>
+    <col width="26" customWidth="1" min="16" max="16"/>
+    <col width="26" customWidth="1" min="17" max="17"/>
+    <col width="26" customWidth="1" min="18" max="18"/>
+    <col width="26" customWidth="1" min="19" max="19"/>
+    <col width="26" customWidth="1" min="20" max="20"/>
+    <col width="26" customWidth="1" min="21" max="21"/>
+    <col width="26" customWidth="1" min="22" max="22"/>
+    <col width="26" customWidth="1" min="23" max="23"/>
+    <col width="26" customWidth="1" min="24" max="24"/>
+    <col width="26" customWidth="1" min="25" max="25"/>
+    <col width="26" customWidth="1" min="26" max="26"/>
+    <col width="26" customWidth="1" min="27" max="27"/>
+    <col width="26" customWidth="1" min="28" max="28"/>
+    <col width="26" customWidth="1" min="29" max="29"/>
+    <col width="26" customWidth="1" min="30" max="30"/>
+    <col width="26" customWidth="1" min="31" max="31"/>
+    <col width="26" customWidth="1" min="32" max="32"/>
+    <col width="26" customWidth="1" min="33" max="33"/>
   </cols>
   <sheetData>
-    <row r="1" ht="60" customHeight="1">
+    <row r="1" ht="48" customHeight="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Content ID</t>
@@ -5602,42 +5602,42 @@
   <dimension ref="A1:AG41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="45" customWidth="1" min="2" max="2"/>
-    <col width="45" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
-    <col width="28" customWidth="1" min="8" max="8"/>
-    <col width="28" customWidth="1" min="9" max="9"/>
-    <col width="28" customWidth="1" min="10" max="10"/>
-    <col width="28" customWidth="1" min="11" max="11"/>
-    <col width="28" customWidth="1" min="12" max="12"/>
-    <col width="28" customWidth="1" min="13" max="13"/>
-    <col width="28" customWidth="1" min="14" max="14"/>
-    <col width="28" customWidth="1" min="15" max="15"/>
-    <col width="28" customWidth="1" min="16" max="16"/>
-    <col width="28" customWidth="1" min="17" max="17"/>
-    <col width="28" customWidth="1" min="18" max="18"/>
-    <col width="28" customWidth="1" min="19" max="19"/>
-    <col width="28" customWidth="1" min="20" max="20"/>
-    <col width="28" customWidth="1" min="21" max="21"/>
-    <col width="28" customWidth="1" min="22" max="22"/>
-    <col width="28" customWidth="1" min="23" max="23"/>
-    <col width="28" customWidth="1" min="24" max="24"/>
-    <col width="28" customWidth="1" min="25" max="25"/>
-    <col width="28" customWidth="1" min="26" max="26"/>
-    <col width="28" customWidth="1" min="27" max="27"/>
-    <col width="28" customWidth="1" min="28" max="28"/>
-    <col width="28" customWidth="1" min="29" max="29"/>
-    <col width="28" customWidth="1" min="30" max="30"/>
-    <col width="28" customWidth="1" min="31" max="31"/>
-    <col width="28" customWidth="1" min="32" max="32"/>
-    <col width="28" customWidth="1" min="33" max="33"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="13" max="13"/>
+    <col width="26" customWidth="1" min="14" max="14"/>
+    <col width="26" customWidth="1" min="15" max="15"/>
+    <col width="26" customWidth="1" min="16" max="16"/>
+    <col width="26" customWidth="1" min="17" max="17"/>
+    <col width="26" customWidth="1" min="18" max="18"/>
+    <col width="26" customWidth="1" min="19" max="19"/>
+    <col width="26" customWidth="1" min="20" max="20"/>
+    <col width="26" customWidth="1" min="21" max="21"/>
+    <col width="26" customWidth="1" min="22" max="22"/>
+    <col width="26" customWidth="1" min="23" max="23"/>
+    <col width="26" customWidth="1" min="24" max="24"/>
+    <col width="26" customWidth="1" min="25" max="25"/>
+    <col width="26" customWidth="1" min="26" max="26"/>
+    <col width="26" customWidth="1" min="27" max="27"/>
+    <col width="26" customWidth="1" min="28" max="28"/>
+    <col width="26" customWidth="1" min="29" max="29"/>
+    <col width="26" customWidth="1" min="30" max="30"/>
+    <col width="26" customWidth="1" min="31" max="31"/>
+    <col width="26" customWidth="1" min="32" max="32"/>
+    <col width="26" customWidth="1" min="33" max="33"/>
   </cols>
   <sheetData>
-    <row r="1" ht="60" customHeight="1">
+    <row r="1" ht="48" customHeight="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Content ID</t>

</xml_diff>